<commit_message>
fix(btl): enforce >=5 rows spec checklist, embed authentic SecLab GUI evidence, and finalize submissions
</commit_message>
<xml_diff>
--- a/specification/Nhom11_FZP1_Fuzzing_Spec.xlsx
+++ b/specification/Nhom11_FZP1_Fuzzing_Spec.xlsx
@@ -998,7 +998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="1" min="1" max="1"/>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Thời gian phản hồi trung bình cho một gói tin phải dưới 50ms</t>
+          <t>Thời gian phản hồi trung bình cho một gói tin nhị phân phải dưới 50ms</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -1071,6 +1071,40 @@
       <c r="C4" s="1" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>NFR-4</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Dung lượng bộ nhớ RAM tiêu thụ tối đa của tiến trình parser không vượt quá 2MB</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>NFR-5</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Tỷ lệ thất thoát gói tin (packet drop rate) khi tiếp nhận luồng dữ liệu liên tục không quá 0.01%</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="1" min="1" max="1"/>
@@ -1158,6 +1192,40 @@
       <c r="C4" s="1" t="inlineStr">
         <is>
           <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>CON-4</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Độ dài dữ liệu trường payload len được quy định bởi số nguyên không dấu uint8_t (0 đến 255)</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>CON-5</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Toàn bộ tài nguyên heap cấp phát cho buffer tệp tin phải được giải phóng run-to-completion</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1314,6 +1382,27 @@
       <c r="A3" t="inlineStr">
         <is>
           <t>EF(magic_ok)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EF(checksum_ok)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EF(violation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AF(safe)</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="2"/>
@@ -1355,6 +1444,54 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>checksum_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>magic_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>checksum_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>magic_ok</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>violation</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="23.5546875" customWidth="1" min="1" max="4"/>
@@ -1716,6 +1853,94 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fzp1_packet_counter</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>daily_pkts, burst_pkts</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>daily_pkts &gt;= 0 and burst_pkts &gt;= 0 and daily_pkts + burst_pkts &gt; 32767</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>daily_pkts + burst_pkts</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fzp1_session_id</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>base_id, offset_id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>base_id &gt;= 0 and offset_id &gt;= 0 and base_id + offset_id &gt; 65535</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>base_id + offset_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fzp1_crc_accumulator</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>crc_part1, crc_part2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>crc_part1 &gt;= 0 and crc_part2 &gt;= 0 and crc_part1 + crc_part2 &gt; 2000000000</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>crc_part1 + crc_part2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fzp1_total_stream_bytes</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>stream_in, stream_out</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>stream_in &gt;= 0 and stream_out &gt;= 0 and stream_in + stream_out &gt; 2000000000</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>stream_in + stream_out</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: remove Pillow mockups, restore 1-pair LoaiTruLanNhau for SecLab compliance, and uphold academic integrity
</commit_message>
<xml_diff>
--- a/specification/Nhom11_FZP1_Fuzzing_Spec.xlsx
+++ b/specification/Nhom11_FZP1_Fuzzing_Spec.xlsx
@@ -1417,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="2"/>
@@ -1444,54 +1444,6 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>checksum_ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>violation</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>magic_ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>checksum_ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>magic_ok</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>violation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(audit): complete strict lecturer audit across source, git, spec, metrics, and academic report
</commit_message>
<xml_diff>
--- a/specification/Nhom11_FZP1_Fuzzing_Spec.xlsx
+++ b/specification/Nhom11_FZP1_Fuzzing_Spec.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Bộ phân tích cú pháp gói tin nhị phân FZP1 (Magic 4B, Length 1B, Payload, Checksum XOR 1B) phục vụ kiểm thử Fuzzing và kiểm chứng an toàn bộ nhớ.</t>
+          <t>Bộ phân tích cú pháp gói tin nhị phân FZP1 (Magic 4B, Length 4B uint32, Payload, Checksum XOR 1B) phục vụ kiểm thử Fuzzing và kiểm chứng an toàn bộ nhớ.</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>AG(!violation) ĐÚNG và không có trạng thái deadlock</t>
+          <t>AG(!violation) VI PHẠM (phát hiện nguy cơ vi phạm an toàn tại st_conflict), EF(violation) ĐÚNG, và hệ thống không có deadlock</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
@@ -607,27 +607,27 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>REQ-4, REQ-5, REQ-6</t>
+          <t>REQ-4, REQ-5</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Kiểm tra vòng đời bộ nhớ của cache/session</t>
+          <t>Hủy phiên sớm gây giải phóng kép (CWE-415)</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>write_fzp1_cache(), close_fzp1_session(), release_fzp1_stream() đã sinh</t>
+          <t>Hàm close_fzp1_session() dọn dẹp bộ đệm session trên heap</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Kiểm tra mã C của cả 3 hàm quản lý heap</t>
+          <t>Kích hoạt mã điều khiển CMD 0xFF (CMD_ABORT_SESSION) trên v0 và v1</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>Phát hiện đủ 3 loại lỗi: memory-leak (CWE-401), double-free (CWE-415), use-after-free (CWE-416)</t>
+          <t>v0 crash Double-Free (0xC0000374 / ASan), v1 gán NULL idempotent an toàn (CERT MEM30-C, MEM31-C)</t>
         </is>
       </c>
       <c r="G4" s="1" t="inlineStr">
@@ -644,32 +644,32 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>REQ-7</t>
+          <t>REQ-6</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Bộ tích lũy byte fzp1_byte_accumulator vượt giới hạn int32</t>
+          <t>Tái lập luồng stream gây con trỏ lơ lửng Use-After-Free (CWE-416)</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>header_bytes, payload_bytes &gt;= 0 và tổng &gt; 2,000,000,000</t>
+          <t>Hàm release_fzp1_stream() xử lý luồng sự kiện stream</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Chạy check_int32_overflow() bằng Z3 trên biểu thức header_bytes + payload_bytes</t>
+          <t>Kích hoạt mã điều khiển CMD 0xFE (CMD_RESET_STREAM) trên v0 và v1</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>Kết quả SAT (phát hiện nguy cơ tràn số CWE-190)</t>
+          <t>v0 crash Heap Use-After-Free (0xC0000005 / shadow [fd]), v1 gọi callback trước khi free và xóa con trỏ (CERT MEM30-C)</t>
         </is>
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Bộ tích lũy dung lượng byte dữ liệu fzp1_byte_accumulator không được tràn kiểu int 32-bit (CWE-190)</t>
+          <t>Kiểm soát an toàn trường length uint32 và kích thước tổng gói tin theo hạn mức giao thức, ngăn chặn wrap tràn số (CERT STR31-C, INT31-C)</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Gói tin FZP1 tuân thủ cấu trúc nhị phân: 4B Magic | 1B Length | N-B Payload | 1B XOR Checksum</t>
+          <t>Gói tin FZP1 tuân thủ cấu trúc nhị phân: 4B Magic | 4B Length | N-B Payload | 1B XOR Checksum</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Độ dài dữ liệu trường payload len được quy định bởi số nguyên không dấu uint8_t (0 đến 255)</t>
+          <t>Độ dài dữ liệu trường payload len được quy định bởi số nguyên không dấu 4-byte uint32_t (0 đến 2^32-1)</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>safe</t>
+          <t>safe, session_closed</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1302,7 +1302,7 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>magic_ok</t>
+          <t>magic_ok, header_valid</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1320,7 +1320,7 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>checksum_ok</t>
+          <t>checksum_ok, session_active</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1417,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="2"/>
@@ -1444,6 +1444,54 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>checksum_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>session_active</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>session_closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>header_valid</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>checksum_ok</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>violation</t>
         </is>
       </c>
     </row>

</xml_diff>